<commit_message>
Update news list: 2026-09-08
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2034,6 +2034,72 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026.09.07 10:41</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>대구시, ‘대구10미데이’로 지역 향토음식 매력 알린다</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30758</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026.09.07 10:36</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>구미시, 추석 앞두고 식품안전 점검 강화…311개소 집중 점검</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30756</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026.09.07 09:09</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>충북도, 외식·숙박업소 가격표시 집중 단속…새 기준 7월·9월 시행</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30762</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-11
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2100,6 +2100,28 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026.09.09 16:30</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>동대문구, 가을 나들이철 먹거리 안전 챙긴다…식품업소 30곳 점검</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30786</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-12
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2122,6 +2122,28 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026.09.11 15:57</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>영암방문의 해 대비 일반음식점 시설개선 지원한다</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30792</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-16
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2144,6 +2144,28 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026.09.15 10:12</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>임실군, ‘임실N치즈축제’ 대비 음식점 식품위생 특별 점검 실시</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30811</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-17
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2166,6 +2166,50 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026.09.16 17:39</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>"음식에서 돌 나왔다" 치아 깨진척 합의금 요구</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30832</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026.09.16 10:04</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>성남시, 음식점 주방 후드 청소비 지원 기준 30년→10년</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30828</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-22
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2210,6 +2210,28 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026.09.19 09:17</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>청주시, 반려동물 동반 음식점 위생용품 구입비 지원</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30842</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-28
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D82"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2232,6 +2232,28 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026.09.28 09:45</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>삼척시, ‘2026년 모범음식점’ 60개소 지정 추진</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30862</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-09-29
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D83"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2254,6 +2254,28 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026.09.22 15:59</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>영천축제, 강변공원서 10월 2일 개최…전시·체험·야외식당 등 다양한 행사 풍성</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30866</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-01
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2276,6 +2276,28 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026.09.30 09:25</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>'2026 광주미식주간' 10월 2일 개막…71개 식당 최대 20% 할인·도보여행 운영</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30872</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-02
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2298,6 +2298,72 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026.10.01 13:45</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>속초시, 지역 대표 ‘모범음식점’ 찾는다… 10월 16일까지 신청 접수</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30896</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026.10.01 13:39</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>보령시, 식품안심업소 환경개선비 지원으로 안전한 먹거리 환경 조성</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30893</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026.10.01 13:23</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>8월 온라인쇼핑 24조 돌파…배달음식·식료품이 견인</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30890</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-06
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2364,6 +2364,28 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026.10.06 09:28</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>소비생활만족도 전국 1위는 ‘대전광역시’</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30908</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-13
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2386,6 +2386,50 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026.10.13 10:46</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>정읍 맛집 후기 올리면 식사비 50% 환급…최대 5만원 상품권 지급</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30946</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026.10.12 14:30</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>전북자치도, 배달 전문 음식점 위생 집중단속</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30932</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-16
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2430,6 +2430,50 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026.10.15 15:56</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>27개 시군구 대표음식 한자리에…‘남도음식문화큰잔치’ 나주서 개막</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30954</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026.10.15 15:53</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>속초시, 소상공인 겨울철 도시가스요금 ‘4개월 분할납부’ 시행</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30952</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-21
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2474,6 +2474,72 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026.10.20 14:08</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>'별점' 매겨 관리…정부 지정 해외 한식당 1000곳으로</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30966</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026.10.19 15:06</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>종로구, 운현궁에 임금님 수라상 차린다… 24일 전통음식축제</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30972</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026.10.19 09:13</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>진천군, 반려동물 동반 출입 음식점 위생용품 지원</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30970</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-22
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2540,6 +2540,50 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026.10.21 15:48</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>‘진안으로 GO! 음식으로 ONE!’ ‘2026 진안고원푸드페스타’ 24~25일 개막!</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30987</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026.10.21 15:45</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2026년 김천시 소상공인 온라인 마케팅 홍보비용 선착순 지원</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30983</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-27
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D98"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2584,6 +2584,28 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026.10.23 11:28</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>강북구, 음식물류 폐기물 다량배출사업장 지도·점검…30일까지</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=30989</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update news list: 2026-10-30
</commit_message>
<xml_diff>
--- a/kfood_news_list.xlsx
+++ b/kfood_news_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2606,6 +2606,50 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026.10.29 09:01</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>"5만원 이상 사면 라면까지"…청주 음식·전통주 맛보고 체험하는 미식 페스타 열린다</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=31022</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026.10.29 08:57</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>제천시, 반려동물 동반 음식점 위생용품 지원…최대 50만원 지급</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>http://www.kfoodtimes.com/news/articleView.html?idxno=31020</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>